<commit_message>
Actualizacion automatica del mapa (2026-05-02 09:53:33)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Magartel.xlsx
+++ b/mapa_interactivo_Magartel.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Magartel" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Magartel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,82 +417,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Caso</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Titulo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Direccion</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Comuna</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Empresa</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Permiso</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>OT</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Coordenada_X</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Coordenada_Y</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Operacion</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>PD</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>N2</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-02 10:08:17)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Magartel.xlsx
+++ b/mapa_interactivo_Magartel.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,7 +544,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">03936328 </t>
+        </is>
+      </c>
       <c r="K2" t="n">
         <v>-58.376816</v>
       </c>
@@ -567,6 +571,376 @@
         </is>
       </c>
       <c r="P2" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>9029</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PEÑA 3161 / Buzon / TELECOM ARGENTINA S.A / Buzon / TELECOM ARGENTINA S.A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>4/23/2026</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PEÑA 3161</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Armario</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>-58.406522</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-34.58509</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Recoleta</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>AGU-J</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S00141694</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SANCHEZ DE BUSTAMANTE 2450 / Buzon / TELECOM ARGENTINA S.A.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>4/23/2026</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SANCHEZ DE BUSTAMANTE 2450</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Armario</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="n">
+        <v>-58.403295</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-34.585041</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Recoleta</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>AGU-H</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S00435449</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>387 SANTIAGO DEL ESTERO - RECLAMO TAPA DESNIVELADA S00435449/26</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>4/27/2026</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SANTIAGO DEL ESTERO 387</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Camara DV</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>-58.384719</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-34.613116</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>CEN-F</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>S00504953</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3418 BENITO JUAREZ - RECLAMO BROCAL ROTO S00504953/26</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>4/27/2026</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BENITO JUAREZ 3418</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Camara DV</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>-58.514869</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-34.60897</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>DEV-E</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>S00507289</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>215 AV RAUL SCALABRINI ORTIZ - URGENTE TAPA ROTA S00507289/26</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>4/27/2026</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AV RAUL SCALABRINI ORTIZ 215</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Camara DV</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>-58.439714</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-34.600565</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>VCR-J</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-05 07:23:21)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Magartel.xlsx
+++ b/mapa_interactivo_Magartel.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,7 +622,11 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
       <c r="K3" t="n">
         <v>-58.406522</v>
       </c>
@@ -696,7 +700,11 @@
           <t>Si</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
       <c r="K4" t="n">
         <v>-58.403295</v>
       </c>
@@ -770,7 +778,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
       <c r="K5" t="n">
         <v>-58.384719</v>
       </c>
@@ -844,7 +856,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
       <c r="K6" t="n">
         <v>-58.514869</v>
       </c>
@@ -918,7 +934,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
       <c r="K7" t="n">
         <v>-58.439714</v>
       </c>
@@ -941,6 +961,84 @@
         </is>
       </c>
       <c r="P7" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SOLICITUD DE CONTINGENCIA CABILDO AV. 1953, CABA EC MAGARTEL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5/4/2026</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>AV CABILDO 1953</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Camara DV</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>-58.455366</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-34.563394</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>BLO-O</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-01 13:41:11)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Magartel.xlsx
+++ b/mapa_interactivo_Magartel.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,27 +501,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>9029</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>825 MAIPU - PRIORITARIO TAPA ROTA</t>
+          <t>PEÑA 3161 / Buzon / TELECOM ARGENTINA S.A / Buzon / TELECOM ARGENTINA S.A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>4/23/2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MAIPU 825</t>
+          <t>PEÑA 3161</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -531,7 +531,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Camara DV</t>
+          <t>Armario</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -541,19 +541,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">03936328 </t>
+          <t xml:space="preserve">04185322 </t>
         </is>
       </c>
       <c r="K2" t="n">
-        <v>-58.376816</v>
+        <v>-58.406522</v>
       </c>
       <c r="L2" t="n">
-        <v>-34.598397</v>
+        <v>-34.58509</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>RTT-?</t>
+          <t>AGU-J</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -579,12 +579,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>9029</t>
+          <t>S00141694</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PEÑA 3161 / Buzon / TELECOM ARGENTINA S.A / Buzon / TELECOM ARGENTINA S.A</t>
+          <t>SANCHEZ DE BUSTAMANTE 2450 / Buzon / TELECOM ARGENTINA S.A.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PEÑA 3161</t>
+          <t>SANCHEZ DE BUSTAMANTE 2450</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -624,14 +624,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>PENDIENTE ADMIN</t>
+          <t xml:space="preserve">04185446 </t>
         </is>
       </c>
       <c r="K3" t="n">
-        <v>-58.406522</v>
+        <v>-58.403295</v>
       </c>
       <c r="L3" t="n">
-        <v>-34.58509</v>
+        <v>-34.585041</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>AGU-J</t>
+          <t>AGU-H</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -657,27 +657,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S00141694</t>
+          <t>S00435449</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SANCHEZ DE BUSTAMANTE 2450 / Buzon / TELECOM ARGENTINA S.A.</t>
+          <t>387 SANTIAGO DEL ESTERO - RECLAMO TAPA DESNIVELADA S00435449/26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>4/23/2026</t>
+          <t>4/27/2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SANCHEZ DE BUSTAMANTE 2450</t>
+          <t>SANTIAGO DEL ESTERO 387</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Armario</t>
+          <t>Camara DV</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -706,14 +706,14 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>-58.403295</v>
+        <v>-58.384719</v>
       </c>
       <c r="L4" t="n">
-        <v>-34.585041</v>
+        <v>-34.613116</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>AGU-H</t>
+          <t>CEN-F</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -735,27 +735,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S00435449</t>
+          <t>S00545181</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>387 SANTIAGO DEL ESTERO - RECLAMO TAPA DESNIVELADA S00435449/26</t>
+          <t>124 CHACABUCO - RECLAMO TAPA DESNIVELADA S00545181/26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>4/27/2026</t>
+          <t>5/11/2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SANTIAGO DEL ESTERO 387</t>
+          <t>CHACABUCO 124</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -778,16 +778,12 @@
           <t>No</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
-        <v>-58.384719</v>
+        <v>-58.376288</v>
       </c>
       <c r="L5" t="n">
-        <v>-34.613116</v>
+        <v>-34.609552</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -801,7 +797,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>CEN-F</t>
+          <t>RTT-?</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -813,27 +809,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S00504953</t>
+          <t>CA0001</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3418 BENITO JUAREZ - RECLAMO BROCAL ROTO S00504953/26</t>
+          <t>CAMARETAS A REPARAR JARAMILLO 2790</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4/27/2026</t>
+          <t>5/12/2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>BENITO JUAREZ 3418</t>
+          <t>JARAMILLO 2790</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -853,7 +849,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -862,14 +858,14 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>-58.514869</v>
+        <v>-58.472378</v>
       </c>
       <c r="L6" t="n">
-        <v>-34.60897</v>
+        <v>-34.549992</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -879,7 +875,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>DEV-E</t>
+          <t>COG-M</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -891,27 +887,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>S00507289</t>
+          <t>CA0002</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>215 AV RAUL SCALABRINI ORTIZ - URGENTE TAPA ROTA S00507289/26</t>
+          <t>SOLICITUD DE CONTINGENCIA LARRALDE 2811 EC MAGARTEL</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>4/27/2026</t>
+          <t>5/12/2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AV RAUL SCALABRINI ORTIZ 215</t>
+          <t>LARRALDE 2811</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -931,7 +927,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Si</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -940,14 +936,14 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>-58.439714</v>
+        <v>-58.472156</v>
       </c>
       <c r="L7" t="n">
-        <v>-34.600565</v>
+        <v>-34.551101</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -957,7 +953,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>VCR-J</t>
+          <t>COG-M</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -969,76 +965,388 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>CA00004</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SOLICITUD DE CONTINGENCIA CABILDO AV. 1953, CABA EC MAGARTEL</t>
+          <t>SOLICITUD DE CONTINGENCIA CONESA 3398 EC MAGARTEL</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>5/4/2026</t>
+          <t>5/12/2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AV CABILDO 1953</t>
+          <t>CONESA 3398</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Camara DV</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>-58.472077</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-34.553986</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>COG-L</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CA0005</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SOLICITUD DE CONTINGENCIA M.PEDRAZA 2639 EC MAGARTEL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>5/12/2026</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MANUELA PEDRAZA 2639</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Camara DV</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>-58.468431</v>
+      </c>
+      <c r="L9" t="n">
+        <v>-34.552835</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>COG-L</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CA00006</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>REPARAR TAPAS PRIORIDAD JARAMILLO 2717</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5/12/2026</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>JARAMILLO 2717</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Camara DV</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>-58.471987</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-34.549696</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>COG-M</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Marco y Tapa Camareta-Cramer 3868-Desmonte Nuñez A48 Etapa 2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5/19/2026</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CRAMER 3868</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>13</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Camara DV</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Magartel</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>PENDIENTE ADMIN</t>
         </is>
       </c>
-      <c r="K8" t="n">
-        <v>-58.455366</v>
-      </c>
-      <c r="L8" t="n">
-        <v>-34.563394</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Colegiales</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
+      <c r="K11" t="n">
+        <v>-58.474587</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-34.548784</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
         <is>
           <t>Capital Norte</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>BLO-O</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>COG-P</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>900009981310</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2351 BORGES, JORGE LUIS - PRIORITARIO TAPA FALTANTE 900009981310</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>5/20/2026</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BORGES, JORGE LUIS 2351</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Camara DV</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Magartel</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>-58.422465</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-34.583308</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>VCR-Q</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>